<commit_message>
Update parsed FINN Vega data
</commit_message>
<xml_diff>
--- a/data/finn_vega.xlsx
+++ b/data/finn_vega.xlsx
@@ -577,7 +577,11 @@
           <t>ANNONSE_001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>4 solgt - kun 2 igjen!</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Nordbohus - Bernhard Olsen AS</t>
@@ -623,7 +627,11 @@
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Tittel hentet fra statusmerke - kontroller manuelt</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -728,7 +736,7 @@
         <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>762</v>
+        <v>108</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>248762</v>

</xml_diff>